<commit_message>
Customize WGR landing and quiz consultation copy
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/incoming/WGR_Store_Data.xlsx
+++ b/incoming/WGR_Store_Data.xlsx
@@ -799,12 +799,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Northeast Wisconsin's #1 furniture &amp; mattress retailer since 1946</t>
+          <t>Serving Northeast Wisconsin since 1946 — proudly employee-owned</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>EST. 1946 - EMPLOYEE-OWNED - WISCONSIN</t>
+          <t>EST. 1946 · EMPLOYEE-OWNED · NORTHEAST WISCONSIN</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -846,27 +846,27 @@
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>WG&amp;R Sleep Shop</t>
+          <t>WG&amp;R Sleep Consultation</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>Let's find your</t>
+          <t>Let's find the mattress</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>best night's sleep</t>
+          <t>made for how you sleep</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Answer a few quick questions and we'll match you to the right mattress - backed by our </t>
+          <t xml:space="preserve">Answer a few questions and our sleep specialists will match you to the right mattress — proudly </t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>125-Night Sleep Guarantee</t>
+          <t>employee-owned in Northeast Wisconsin since 1946</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Start the Sleep Quiz</t>
+          <t>Start My Sleep Consultation</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>Takes about 2 minutes</t>
+          <t>About 2 minutes, no pressure</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr"/>

</xml_diff>

<commit_message>
Enable WG&R bilingual experience and refine showroom results
</commit_message>
<xml_diff>
--- a/incoming/WGR_Store_Data.xlsx
+++ b/incoming/WGR_Store_Data.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brands" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mattresses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Accessories" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SalesNotes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mattresses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SalesNotes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -730,7 +730,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>en,es</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL27"/>
+  <dimension ref="A1:AT27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1193,62 +1193,102 @@
       </c>
       <c r="AA1" t="inlineStr">
         <is>
+          <t>differentiator1Title</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>differentiator1Detail</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>differentiator2Title</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>differentiator2Detail</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>displayBadges (ES)</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>highlight (ES)</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>reason_cooling (ES)</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>reason_pressureRelief (ES)</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>reason_motionIsolation (ES)</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>reason_support (ES)</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>reason_plush (ES)</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>reason_medium (ES)</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>reason_firm (ES)</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>reason_durability (ES)</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>reason_default (ES)</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>topPickReason (ES)</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>differentiator1Title (ES)</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>differentiator1Detail (ES)</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>differentiator2Title (ES)</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>differentiator2Detail (ES)</t>
         </is>
       </c>
     </row>
@@ -1339,14 +1379,86 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Espuma viscoelástica|Alivio de presión|Medio</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Se adapta a tu cuerpo para un alivio profundo de presión</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>Espuma viscoelástica que se adapta al cuerpo para un alivio profundo de presión.</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>El material TEMPUR se adapta a ti para aliviar la presión y reducir la transferencia de movimiento.</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>Contorno TEMPUR de adaptación lenta</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>Se ajusta de cerca al cuerpo en vez de empujar como una cama con más rebote.</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Sensación de espuma que absorbe movimiento</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Mantiene más silencioso el movimiento de la pareja que los diseños con resortes.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1435,14 +1547,86 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Enfriamiento|Híbrido|Medio</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Confort adaptable con soporte híbrido y frescura toda la noche</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>Confort de espuma adaptable con respuesta híbrida y frescura toda la noche.</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>Duerme más fresco con confort TEMPUR y soporte híbrido sensible.</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>Contorno TEMPUR con elevación de resortes</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>Combina alivio de presión lento arriba con movimiento más fácil gracias a la base híbrida.</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>Enfriamiento enfocado Breeze</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>Diseñado para sentirse más fresco que la espuma tradicional de contorno profundo.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1531,14 +1715,86 @@
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Enfriamiento|Firme|Alivio de presión</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Nuestro TEMPUR más fresco firme y con buen soporte</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Nuestra opción más fresca con confort firme y soporte completo.</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Nuestro TEMPUR más fresco con confort firme y soporte durante toda la noche.</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>La sensación Breeze más firme</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>Una superficie estable de 7/10 ofrece menos hundimiento sin perder el contorno TEMPUR.</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>Máximo enfriamiento Breeze</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>La construcción enfocada en frescura es el principal avance dentro de la línea Breeze.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1627,14 +1883,86 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Firme|Soporte de resortes|Duradero</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Soporte firme de resortes hecho a mano y diseñado para durar</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>Soporte firme y duradero de resortes hecho a mano para brindar confort prolongado.</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Los resortes de precisión brindan soporte firme y duradero.</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>Respuesta de resortes hecha a mano</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>Los resortes de precisión crean una sensación estructurada con más elevación que la espuma.</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>Enfoque firme y duradero</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>Diseñado para conservar una sensación estable en vez de un hundimiento profundo.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1723,14 +2051,86 @@
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Resortes de lujo|Medio|Duradero</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>Lujo artesanal suave en la superficie y apoyado por debajo</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Resortes y espumas premium equilibrados para un lujo suave y con buen soporte.</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Resortes y espumas premium hechos a mano para un lujo equilibrado y duradero.</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Equilibrio de lujo suave y apoyado</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>Las capas de confort suavizan el primer contacto mientras los resortes mantienen el apoyo.</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>Construcción estilo reliquia</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Espumas y resortes premium crean una sensación sustancial y una construcción duradera.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1819,14 +2219,86 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Látex Talalay|Suave|Duradero</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Confort suave de látex completo con durabilidad excepcional</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Suavidad de látex Talalay natural con durabilidad excepcional.</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>Confort suave de látex completo con una garantía que destaca.</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>Flotación de látex Talalay</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>Se siente elástico y responde al instante sin el hundimiento lento de la espuma viscoelástica.</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Durabilidad de látex completo</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Usa látex resistente en toda la estructura de confort y no solo como una capa delgada.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1915,14 +2387,86 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Rejilla GelFlex|Enfriamiento|Sensible</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Rejilla GelFlex premium fresca sensible y sin presión</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>La rejilla GelFlex premium de Purple ofrece una sensación fresca y sensible con alivio de presión.</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>La rejilla premium de Purple brinda una sensación fresca y sensible sin presión.</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Respuesta de rejilla GelFlex</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>La rejilla cede justo bajo los puntos de presión y mantiene apoyo alrededor.</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>Sensación flotante y abierta</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Envuelve menos que la espuma y permite moverse con mayor facilidad.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2011,14 +2555,86 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Resortes embolsados|Medio|Aislamiento de movimiento</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Sensación media de lujo con soporte premium de resortes</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>Confort medio de lujo sobre soporte premium de resortes embolsados.</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>Sensación media de lujo sobre el soporte premium de resortes embolsados Beautyrest.</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>Centro premium de resortes embolsados</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>Los resortes individuales dan apoyo definido y limitan el movimiento a través de la cama.</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>Acolchado medio de lujo</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Agrega una superficie más refinada sin perder la respuesta de los resortes.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2107,14 +2723,86 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Ajuste inteligente|Firmeza doble|Zonas</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Firmeza inteligente ajustable por lado a tu manera</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>Una cama inteligente que ajusta la firmeza de cada lado a cada persona.</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>Ajusta la firmeza de cada lado con soporte inteligente controlado por aplicación.</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>Firmeza independiente por lado</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>Cada persona puede ajustar su lado sin comprometerse con una sola sensación compartida.</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Ajuste controlado por aplicación</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>La firmeza puede cambiar después de la compra cuando evolucionen las preferencias.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2199,14 +2887,86 @@
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Rejilla GelFlex|Enfriamiento|Sensible</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>La rejilla Purple original fresca sensible y adaptable</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>La rejilla Purple original ofrece frescura respuesta y adaptación.</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>Confort fresco y sensible de rejilla que se adapta mientras te mueves.</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>Experiencia GelFlex original</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>La rejilla se dobla bajo los puntos de presión y recupera su forma al moverte.</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>Perfil Purple más sencillo</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>Ofrece la sensación flotante de la rejilla sin una construcción de lujo más gruesa.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2295,14 +3055,86 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>Híbrido de rejilla|Firme|Sensible</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Rejilla firme sobre resortes con flujo de aire</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>Soporte firme de rejilla sobre resortes con ventilación y alivio de presión.</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Soporte firme de rejilla sobre resortes con ventilación y alivio de presión.</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>Rejilla firme sobre resortes</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>Combina la superficie flexible de Purple con el empuje más fuerte de una base híbrida.</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>Apoyo ventilado y sensible</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>La rejilla abierta y los resortes se sienten menos encerrados que una espuma firme y densa.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2391,14 +3223,86 @@
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>Enfriamiento|Zonas|Híbrido</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Duerme más fresco con soporte por zonas</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>Duerme más fresco con soporte por zonas pensado para quienes sienten calor.</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Duerme más fresco con soporte por zonas para quienes sienten calor.</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>Híbrido enfocado en enfriamiento</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>Su propósito principal es reducir el calor sin perder una sensación fácil para moverse.</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>Distribución de apoyo por zonas</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>Diferentes áreas amortiguan los puntos de presión y estabilizan el centro del cuerpo.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2487,14 +3391,86 @@
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>Híbrido|Enfriamiento|Medio</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Confort híbrido equilibrado con frescura</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>Confort híbrido equilibrado y fresco a un precio accesible.</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Confort híbrido equilibrado y fresco a un precio accesible.</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>Híbrido equilibrado para diario</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>No envuelve demasiado ni se siente muy firme; busca una sensación intermedia fácil.</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>Elevación de resortes accesible</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>Ofrece el movimiento de un híbrido sin subir a una construcción premium.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2583,14 +3559,86 @@
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Híbrido|Medio|Soporte</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Confort híbrido Sealy confiable</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>Soporte híbrido Sealy confiable para un confort diario equilibrado.</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Híbrido Sealy confiable ajustado para un confort equilibrado toda la noche.</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>Sensación híbrida Sealy familiar</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>Una superficie media sobre apoyo sensible se entiende rápidamente al probarla.</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>Simplicidad enfocada en apoyo</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Prioriza alineación y movimiento confiables sobre tecnología inteligente o de rejilla.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2679,14 +3727,86 @@
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
-      <c r="AL16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>Híbrido|Firme|Soporte</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Soporte híbrido firme para mantener la alineación</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>Soporte híbrido firme que ayuda a mantener la columna alineada.</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Soporte híbrido firme que ayuda a mantener la columna alineada.</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Perfil Posturepedic firme</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>Una superficie de 7/10 mantiene el cuerpo más encima del colchón que dentro de él.</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>Construcción híbrida estable</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Combina capas firmes con resortes para una respuesta más estable que la espuma firme sola.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2775,14 +3895,86 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr"/>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
-      <c r="AL17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Resortes embolsados|Firme|Aislamiento de movimiento</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>Soporte firme de resortes con sensación de lujo</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>Soporte firme de resortes embolsados con una verdadera sensación de lujo.</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>Soporte firme de resortes embolsados Beautyrest con sensación de lujo.</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>Sensación firme de resortes Beautyrest</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>Ofrece un empuje fuerte con la respuesta familiar de resortes premium.</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>Control de movimiento embolsado</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>Los resortes individuales se mueven con más independencia que una unidad tradicional conectada.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2867,14 +4059,86 @@
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr"/>
-      <c r="AL18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>Hecho en Wisconsin|Suave|Alivio de presión</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Confort suave hecho a mano en Wisconsin</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>Confort suave que alivia la presión y está hecho a mano en Wisconsin.</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>Confort suave Astor Park que alivia la presión y está hecho a mano en Wisconsin.</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>Suavidad hecha a mano en Wisconsin</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>Fabricado localmente con una superficie muy suave de 3/10 para quien quiere acolchado inmediato.</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>Mayor alivio en puntos de presión</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>Permite que hombros y caderas bajen más que en las opciones medias y firmes.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2959,14 +4223,86 @@
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
-      <c r="AK19" t="inlineStr"/>
-      <c r="AL19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>Hecho en Wisconsin|Firme|Duradero</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Soporte firme hecho a mano en Wisconsin</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>Confort firme y con buen soporte hecho a mano en Wisconsin.</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Firmeza artesanal de Wisconsin con soporte confiable toda la noche.</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>Firmeza hecha a mano en Wisconsin</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>Fabricado localmente con una superficie estable de 7/10 y poco hundimiento inicial.</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>Apoyo enfocado en durabilidad</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>Destaca una construcción firme y directa sobre capas adicionales de suavidad.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3055,14 +4391,86 @@
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
-      <c r="AF20" t="inlineStr"/>
-      <c r="AG20" t="inlineStr"/>
-      <c r="AH20" t="inlineStr"/>
-      <c r="AI20" t="inlineStr"/>
-      <c r="AJ20" t="inlineStr"/>
-      <c r="AK20" t="inlineStr"/>
-      <c r="AL20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>Híbrido|Enfriamiento|Aislamiento de movimiento</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Confort híbrido fresco para parejas</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>Confort híbrido fresco con buen aislamiento de movimiento para parejas.</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>Confort híbrido fresco y aislamiento de movimiento para parejas.</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>Híbrido fresco para parejas</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>Combina ventilación y control de movimiento para parejas que duermen con calor o se despiertan.</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>Equilibrio de espuma y resortes</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>Ofrece algo de contorno arriba y conserva el movimiento más fácil de un híbrido.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3151,14 +4559,86 @@
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr"/>
       <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="inlineStr"/>
-      <c r="AF21" t="inlineStr"/>
-      <c r="AG21" t="inlineStr"/>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
-      <c r="AK21" t="inlineStr"/>
-      <c r="AL21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>Espuma viscoelástica|Enfriamiento|Medio</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Confort fresco de espuma a un precio accesible</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>Confort fresco de espuma en caja que cuida el presupuesto.</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>Confort fresco de espuma en caja que cuida el presupuesto.</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>Inicio sencillo de espuma</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>Ofrece contorno cercano y una superficie silenciosa sin el rebote de resortes.</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>Enfriamiento con buen valor</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>Agrega materiales para controlar el calor dentro del nivel más accesible.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3247,14 +4727,86 @@
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
-      <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr"/>
-      <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
-      <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>Híbrido|Enfriamiento|Medio</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Respuesta híbrida fresca a precio inicial</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>Respuesta híbrida y frescura a un precio inicial accesible.</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>Respuesta híbrida y frescura a un precio inicial accesible.</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>Elevación híbrida de entrada</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>Los resortes facilitan girarse y levantarse más que en el Classic de espuma.</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>Frescura a precio inicial</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>Combina una superficie más fresca con apoyo híbrido en el nivel de entrada.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3343,14 +4895,86 @@
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
-      <c r="AK23" t="inlineStr"/>
-      <c r="AL23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>Híbrido|Medio firme|Buen valor</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Híbrido suave y firme con sensación superior a su precio</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>Un híbrido suave y firme que se siente superior a su precio.</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>Un híbrido suave y firme que se siente muy superior a su precio.</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>Contraste suave y firme</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>El acolchado suaviza la parte superior mientras la base híbrida de 6/10 mantiene empuje.</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>Sensación de valor más sustancial</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>Busca una impresión más sólida y terminada que un colchón inicial básico.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3435,14 +5059,86 @@
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
-      <c r="AF24" t="inlineStr"/>
-      <c r="AG24" t="inlineStr"/>
-      <c r="AH24" t="inlineStr"/>
-      <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" t="inlineStr"/>
-      <c r="AK24" t="inlineStr"/>
-      <c r="AL24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>Suave|Acolchado|Buen valor</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Confort suave y confiable a un precio accesible</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>Confort suave y accesible de una marca reconocida.</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>Confort suave y accesible de una marca conocida.</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>Sensación Sealy suave de entrada</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>Una superficie de 3/10 da suavidad inmediata sin la complejidad del nivel premium.</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>Alivio de presión sencillo</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>Usa acolchado suave y directo para hombros y caderas a un precio accesible.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3527,14 +5223,86 @@
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
-      <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
-      <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>Hecho en Wisconsin|Firme|Buen valor</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Soporte firme hecho en Wisconsin a un gran valor</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>Soporte firme hecho en Wisconsin a un precio accesible.</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>Soporte firme hecho en Wisconsin a un precio ideal para una habitación de visitas.</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>Valor firme hecho en Wisconsin</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>Fabricado localmente con una sensación estable de 7/10 y una propuesta de apoyo directa.</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>Simplicidad para habitación de visitas</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>Prioriza firmeza confiable y precio sobre capas de enfriamiento o lujo.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3623,14 +5391,86 @@
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
       <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr"/>
-      <c r="AI26" t="inlineStr"/>
-      <c r="AJ26" t="inlineStr"/>
-      <c r="AK26" t="inlineStr"/>
-      <c r="AL26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>Euro Top|Medio|Buen valor</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Euro top suave sobre soporte confiable</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>Confort suave de euro top sobre soporte confiable de resortes.</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>Confort suave de euro top sobre soporte confiable de resortes.</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>Primera impresión Euro Top</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>El acolchado cosido crea una superficie más suave sobre un centro de apoyo medio.</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>Respuesta tradicional de resortes</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>Se siente más familiar y elástico que un colchón de espuma de contorno lento.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3719,14 +5559,86 @@
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr"/>
-      <c r="AH27" t="inlineStr"/>
-      <c r="AI27" t="inlineStr"/>
-      <c r="AJ27" t="inlineStr"/>
-      <c r="AK27" t="inlineStr"/>
-      <c r="AL27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>Híbrido|Medio|Buen valor</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>Confort híbrido mejorado con más espuma y soporte</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>Los materiales transpirables ayudan a disipar el calor.</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>La superficie amortigua hombros y caderas para aliviar puntos de presión.</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>Ayuda a reducir la transferencia de movimiento entre ambos lados de la cama.</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>El sistema de soporte ayuda a mantener el cuerpo alineado.</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>La superficie suave ofrece mayor acolchado y adaptación.</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>La sensación media equilibra suavidad y soporte.</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>La superficie firme ofrece apoyo estable con menos hundimiento.</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Los materiales resistentes están diseñados para conservar su sensación.</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>Más espuma y soporte que el híbrido de entrada.</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>Más espuma y soporte que el híbrido de entrada para ofrecer un poco más.</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>Confort híbrido mejorado</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>Agrega más acolchado y apoyo que el híbrido DreamCloud de entrada.</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>Respuesta intermedia</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>Mantiene una sensación media con elevación de resortes sin hundimiento profundo ni empuje firme.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3739,7 +5651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3825,25 +5737,30 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>Score: Reflux</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Score: Premium</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Score: Position Side</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Score: Position Back</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Score: Position Stomach</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Score: Allergies</t>
         </is>
@@ -3860,13 +5777,21 @@
           <t>BedTech Relax Lifestyle Base</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Base Ajustable BedTech Relax Lifestyle</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Foundations &amp; Support</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bases y Soportes</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>adjustable</t>
@@ -3880,7 +5805,11 @@
           <t>Adjustable power base with head &amp; foot articulation, wireless remote, and memory positions.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Base eléctrica ajustable con elevación de cabeza y pies, control inalámbrico y posiciones de memoria.</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>images/accessories/base-bedtech-relax.jpg</t>
@@ -3901,12 +5830,15 @@
         <v>4</v>
       </c>
       <c r="Q2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R2" t="n">
         <v>3</v>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3919,13 +5851,21 @@
           <t>TEMPUR-Ergo Smart 3.0 Base</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Base TEMPUR-Ergo Smart 3.0</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Foundations &amp; Support</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Bases y Soportes</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>adjustable</t>
@@ -3939,7 +5879,11 @@
           <t>Smart adjustable base with app control, head &amp; foot adjustment, and sleep tracking.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Base inteligente ajustable con control por aplicación, elevación de cabeza y pies, y seguimiento del sueño.</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>images/accessories/base-tempur-ergo-smart.jpg</t>
@@ -3960,12 +5904,15 @@
         <v>4</v>
       </c>
       <c r="Q3" t="n">
+        <v>4</v>
+      </c>
+      <c r="R3" t="n">
         <v>3</v>
       </c>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3978,13 +5925,21 @@
           <t>Purple Premium Plus Smart Base</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Base Inteligente Purple Premium Plus</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Foundations &amp; Support</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Bases y Soportes</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>adjustable</t>
@@ -3998,7 +5953,11 @@
           <t>Smart adjustable base with app control and full head &amp; foot articulation.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Base inteligente ajustable con control por aplicación y articulación completa de cabeza y pies.</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>images/accessories/base-purple-premium-plus.jpg</t>
@@ -4019,12 +5978,15 @@
         <v>4</v>
       </c>
       <c r="Q4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R4" t="n">
         <v>3</v>
       </c>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4037,13 +5999,21 @@
           <t>WG&amp;R Factory Direct Slate Foundation</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Base Slate de WG&amp;R Factory Direct</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Foundations &amp; Support</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Bases y Soportes</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>foundation</t>
@@ -4057,7 +6027,11 @@
           <t>Sturdy standard-height foundation - solid platform support for any mattress.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Base resistente de altura estándar con soporte de plataforma sólida para cualquier colchón.</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>images/accessories/foundation-wgr-slate.jpg</t>
@@ -4080,6 +6054,7 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4092,13 +6067,21 @@
           <t>WG&amp;R Slate Low-Profile Foundation</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Base Slate de Perfil Bajo de WG&amp;R</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Foundations &amp; Support</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bases y Soportes</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>low_profile</t>
@@ -4112,7 +6095,11 @@
           <t>Reduced-height foundation - ideal for taller mattresses or a low-profile look.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Base de menor altura, ideal para colchones altos o para lograr una apariencia de perfil bajo.</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>images/accessories/foundation-wgr-slate-lowpro.jpg</t>
@@ -4135,6 +6122,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4147,13 +6135,21 @@
           <t>WG&amp;R Factory Direct Bunkie Board</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tabla Bunkie de WG&amp;R Factory Direct</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Foundations &amp; Support</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bases y Soportes</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>bunkie</t>
@@ -4167,7 +6163,11 @@
           <t>Slim 2-inch support board for platform and bunk beds.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Tabla delgada de soporte de 2 pulgadas para camas de plataforma y literas.</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>images/accessories/bunkie-wgr.jpg</t>
@@ -4190,6 +6190,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4202,13 +6203,21 @@
           <t>TEMPUR-Breeze ProLo 2.0 Pillow</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Almohada TEMPUR-Breeze ProLo 2.0</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>Pillows</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Almohadas</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>225</v>
@@ -4218,7 +6227,11 @@
           <t>Cooling low-profile TEMPUR pillow for back and stomach sleepers.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Almohada TEMPUR fresca de perfil bajo para quienes duermen boca arriba o boca abajo.</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>images/accessories/pillow-tempur-breeze-prolo.jpg</t>
@@ -4240,13 +6253,14 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" t="n">
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="n">
         <v>2</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>1</v>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4259,13 +6273,21 @@
           <t>TEMPUR-Adapt ProAdjust Pillow</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Almohada TEMPUR-Adapt ProAdjust</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Pillows</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Almohadas</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>125</v>
@@ -4275,7 +6297,11 @@
           <t>Adjustable-fill TEMPUR pillow that customizes to any sleep position.</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Almohada TEMPUR de relleno ajustable que se adapta a cualquier posición para dormir.</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>images/accessories/pillow-tempur-proadjust.jpg</t>
@@ -4294,16 +6320,17 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="n">
-        <v>1</v>
-      </c>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
         <v>1</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4316,13 +6343,21 @@
           <t>Healthy Sleep Cool-Tech Graphite Pillow</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Almohada Healthy Sleep Cool-Tech Graphite</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Pillows</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Almohadas</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>109</v>
@@ -4332,7 +6367,11 @@
           <t>Graphite-infused cooling pillow that draws heat away all night.</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Almohada fresca con grafito que ayuda a disipar el calor durante toda la noche.</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>images/accessories/pillow-cooltech-graphite.jpg</t>
@@ -4353,14 +6392,15 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="n">
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="n">
         <v>1</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>2</v>
       </c>
-      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4373,13 +6413,21 @@
           <t>Purple Waterproof Protector</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Protector Impermeable Purple</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Protectors</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Protectores</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>119</v>
@@ -4389,7 +6437,11 @@
           <t>Waterproof protector that guards your mattress while staying breathable.</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Protector impermeable y transpirable que ayuda a cuidar el colchón.</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>images/accessories/protector-purple-waterproof.jpg</t>
@@ -4397,7 +6449,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>all, allergies</t>
+          <t>all, allergies, spills, everyday</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -4411,7 +6463,8 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="n">
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4426,13 +6479,21 @@
           <t>Healthy Sleep Premium Encasement</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Funda Integral Healthy Sleep Premium</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>Protectors</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Protectores</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>79</v>
@@ -4442,7 +6503,11 @@
           <t>Full-zip encasement - allergen and dust-mite barrier on all six sides.</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Funda integral con cierre que crea una barrera contra alérgenos y ácaros en los seis lados.</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>images/accessories/protector-healthy-sleep-encasement.jpg</t>
@@ -4450,7 +6515,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>allergies, all</t>
+          <t>allergies, all, everyday</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -4464,7 +6529,8 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="n">
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4479,13 +6545,21 @@
           <t>TEMPUR-Protect Breeze Protector</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Protector TEMPUR-Protect Breeze</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>Protectors</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Protectores</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>249</v>
@@ -4495,7 +6569,11 @@
           <t>Cooling protector that adds a breathable layer of protection.</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Protector fresco que agrega una capa transpirable de protección.</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>images/accessories/protector-tempur-breeze.jpg</t>
@@ -4503,7 +6581,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>cooling, hot_sleeper, all</t>
+          <t>cooling, hot_sleeper, all, everyday</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -4520,6 +6598,7 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add WG&R qualification, bilingual, and privacy/CAN-SPAM draft pass
Qualification: true-raw 60% gate (mattresses, accessories, sleep-system
groups), two-choice floor with backfilled "Additional comparison option"
labels carried through results/handoff/email; no scoring-weight changes.

Bilingual: precompute EN/ES profile subtitle, sleep brief, and trial focus
so downstream screens don't inherit the active-render language; trial focus
stored as {en,es}; Spanish archetype leak removed from Guided Trial.

Privacy/CAN-SPAM (DRAFT, pending WG&R approval — gasUrl stays blank):
- Bilingual Privacy & Terms overlay via store-config text/text_es
- Email CAN-SPAM footer (unsubscribe + postal address + privacy contact),
  HTML and plain-text, EN/ES
- Placeholder values clearly marked unverified

Note: store-config privacy fields are hand-added and not yet in the
workbook schema/converter — do not regenerate config before go-live.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/incoming/WGR_Store_Data.xlsx
+++ b/incoming/WGR_Store_Data.xlsx
@@ -833,17 +833,49 @@
           <t>Northeast Wisconsin</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>DreamFinder - Cuestionario del Sueño de WG&amp;R Furniture</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Responde el cuestionario de WG&amp;R Sleep Shop y recibe recomendaciones personalizadas de colchones.</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>DreamFinder - WG&amp;R Furniture</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Sirviendo a Northeast Wisconsin desde 1946 — con orgullo, propiedad de sus empleados</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>PROPIEDAD DE SUS EMPLEADOS · NORTHEAST WISCONSIN · DESDE 1946</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Solo usaremos tu correo para enviarte tus resultados.</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>En stock en WG&amp;R</t>
+        </is>
+      </c>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Northeast Wisconsin</t>
+        </is>
+      </c>
       <c r="AK2" t="inlineStr">
         <is>
           <t>WG&amp;R Sleep Consultation</t>
@@ -884,14 +916,38 @@
           <t>About 2 minutes, no pressure</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>PROPIEDAD DE SUS EMPLEADOS · NORTHEAST WISCONSIN · DESDE 1946</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Northeast Wisconsin,</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>tu tienda del descanso.</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>Responde unas preguntas y revisa tus opciones de colchón con un especialista del descanso de WG&amp;R.</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>Encontrar Mi Opción Ideal</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>Aproximadamente 2 minutos · Sin presión</t>
+        </is>
+      </c>
       <c r="BA2" t="inlineStr">
         <is>
           <t>DreamFinder - WG&amp;R Furniture</t>

</xml_diff>